<commit_message>
Add Profiles sheet with PP2.5, SP2, SP10 figures as native charts
Recreates Figures 3-5 and Tables 2-3 from the source document: pressure
profile PP2.5 and speed profiles SP2/SP10 as scatter-line charts backed by
their time/value data tables.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UUGCHQdTqxssX5bTKDFmqr
</commit_message>
<xml_diff>
--- a/brake_noise_test_procedure.xlsx
+++ b/brake_noise_test_procedure.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Test Procedure" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +42,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -89,7 +98,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -111,11 +120,88 @@
         <color rgb="00808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +244,17 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -232,6 +329,401 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln w="15000">
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="square"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Profiles'!$B$4:$B$6</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Profiles'!$C$4:$C$6</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="12"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Time / s</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="300"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Brake pressure / kPa</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln w="15000">
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="square"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Profiles'!$B$25:$B$32</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Profiles'!$C$25:$C$32</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="60"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Time / s</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="2.5"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Speed / km/h</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln w="15000">
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="square"/>
+            <size val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="4472C4"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Profiles'!$B$48:$B$51</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Profiles'!$C$48:$C$51</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="14"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Time / s</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="12"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Speed / km/h</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -606,10 +1098,10 @@
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
+      <c r="A2" s="16" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
           <t>km/h</t>
@@ -630,9 +1122,9 @@
           <t>kPa</t>
         </is>
       </c>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
+      <c r="I2" s="16" t="n"/>
+      <c r="J2" s="16" t="n"/>
+      <c r="K2" s="16" t="n"/>
     </row>
     <row r="3" ht="118" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -651,14 +1143,14 @@
 (선택 사항) 로터(드럼)와 패드(라이닝)의 두께와 무게를 측정합니다. 테스트 요청에 따라 고정 장치, 예압, 테스트 하드웨어, 마이크 및 가속도계를 철저히 검사합니다. 테스트 설정을 기록하기 위해 디지털 사진을 촬영합니다. 마이크와 가속도계 교정을 수행합니다. 7.3.3항에 따라 냉각 공기를 사용하여 배경 소음 점검을 수행합니다.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
+      <c r="D3" s="17" t="n"/>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="17" t="n"/>
+      <c r="H3" s="17" t="n"/>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="18" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -958,7 +1450,7 @@
           <t>4.2</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n"/>
+      <c r="B10" s="19" t="n"/>
       <c r="C10" s="7" t="n">
         <v>15</v>
       </c>
@@ -1005,7 +1497,7 @@
           <t>4.3</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n"/>
+      <c r="B11" s="16" t="n"/>
       <c r="C11" s="7" t="n">
         <v>9</v>
       </c>
@@ -1187,7 +1679,7 @@
           <t>6.2</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n"/>
+      <c r="B15" s="19" t="n"/>
       <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
@@ -1230,7 +1722,7 @@
           <t>6.3</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n"/>
+      <c r="B16" s="19" t="n"/>
       <c r="C16" s="7" t="n">
         <v>3</v>
       </c>
@@ -1273,7 +1765,7 @@
           <t>6.4</t>
         </is>
       </c>
-      <c r="B17" s="15" t="n"/>
+      <c r="B17" s="19" t="n"/>
       <c r="C17" s="7" t="n">
         <v>3</v>
       </c>
@@ -1316,7 +1808,7 @@
           <t>6.5</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n"/>
+      <c r="B18" s="19" t="n"/>
       <c r="C18" s="7" t="n">
         <v>3</v>
       </c>
@@ -1359,7 +1851,7 @@
           <t>6.6</t>
         </is>
       </c>
-      <c r="B19" s="15" t="n"/>
+      <c r="B19" s="16" t="n"/>
       <c r="C19" s="7" t="n">
         <v>3</v>
       </c>
@@ -1544,7 +2036,7 @@
           <t>8.2</t>
         </is>
       </c>
-      <c r="B23" s="15" t="n"/>
+      <c r="B23" s="19" t="n"/>
       <c r="C23" s="7" t="n">
         <v>9</v>
       </c>
@@ -1591,7 +2083,7 @@
           <t>8.3</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n"/>
+      <c r="B24" s="19" t="n"/>
       <c r="C24" s="7" t="n">
         <v>9</v>
       </c>
@@ -1638,7 +2130,7 @@
           <t>8.4</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n"/>
+      <c r="B25" s="19" t="n"/>
       <c r="C25" s="7" t="n">
         <v>9</v>
       </c>
@@ -1685,7 +2177,7 @@
           <t>8.5</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n"/>
+      <c r="B26" s="19" t="n"/>
       <c r="C26" s="7" t="n">
         <v>9</v>
       </c>
@@ -1732,7 +2224,7 @@
           <t>8.6</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
+      <c r="B27" s="19" t="n"/>
       <c r="C27" s="7" t="n">
         <v>9</v>
       </c>
@@ -1779,7 +2271,7 @@
           <t>8.7</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n"/>
+      <c r="B28" s="16" t="n"/>
       <c r="C28" s="7" t="n">
         <v>9</v>
       </c>
@@ -1968,7 +2460,7 @@
           <t>10.2</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n"/>
+      <c r="B32" s="19" t="n"/>
       <c r="C32" s="7" t="n">
         <v>15</v>
       </c>
@@ -2015,7 +2507,7 @@
           <t>10.3</t>
         </is>
       </c>
-      <c r="B33" s="15" t="n"/>
+      <c r="B33" s="16" t="n"/>
       <c r="C33" s="7" t="n">
         <v>9</v>
       </c>
@@ -2197,7 +2689,7 @@
           <t>12.2</t>
         </is>
       </c>
-      <c r="B37" s="15" t="n"/>
+      <c r="B37" s="19" t="n"/>
       <c r="C37" s="7" t="n">
         <v>3</v>
       </c>
@@ -2240,7 +2732,7 @@
           <t>12.3</t>
         </is>
       </c>
-      <c r="B38" s="15" t="n"/>
+      <c r="B38" s="19" t="n"/>
       <c r="C38" s="7" t="n">
         <v>3</v>
       </c>
@@ -2283,7 +2775,7 @@
           <t>12.4</t>
         </is>
       </c>
-      <c r="B39" s="15" t="n"/>
+      <c r="B39" s="19" t="n"/>
       <c r="C39" s="7" t="n">
         <v>3</v>
       </c>
@@ -2326,7 +2818,7 @@
           <t>12.5</t>
         </is>
       </c>
-      <c r="B40" s="15" t="n"/>
+      <c r="B40" s="19" t="n"/>
       <c r="C40" s="7" t="n">
         <v>3</v>
       </c>
@@ -2369,7 +2861,7 @@
           <t>12.6</t>
         </is>
       </c>
-      <c r="B41" s="15" t="n"/>
+      <c r="B41" s="16" t="n"/>
       <c r="C41" s="7" t="n">
         <v>3</v>
       </c>
@@ -2554,7 +3046,7 @@
           <t>14.2</t>
         </is>
       </c>
-      <c r="B45" s="15" t="n"/>
+      <c r="B45" s="19" t="n"/>
       <c r="C45" s="7" t="n">
         <v>9</v>
       </c>
@@ -2601,7 +3093,7 @@
           <t>14.3</t>
         </is>
       </c>
-      <c r="B46" s="15" t="n"/>
+      <c r="B46" s="19" t="n"/>
       <c r="C46" s="7" t="n">
         <v>9</v>
       </c>
@@ -2648,7 +3140,7 @@
           <t>14.4</t>
         </is>
       </c>
-      <c r="B47" s="15" t="n"/>
+      <c r="B47" s="19" t="n"/>
       <c r="C47" s="7" t="n">
         <v>9</v>
       </c>
@@ -2695,7 +3187,7 @@
           <t>14.5</t>
         </is>
       </c>
-      <c r="B48" s="15" t="n"/>
+      <c r="B48" s="19" t="n"/>
       <c r="C48" s="7" t="n">
         <v>9</v>
       </c>
@@ -2742,7 +3234,7 @@
           <t>14.6</t>
         </is>
       </c>
-      <c r="B49" s="15" t="n"/>
+      <c r="B49" s="19" t="n"/>
       <c r="C49" s="7" t="n">
         <v>9</v>
       </c>
@@ -2789,7 +3281,7 @@
           <t>14.7</t>
         </is>
       </c>
-      <c r="B50" s="15" t="n"/>
+      <c r="B50" s="16" t="n"/>
       <c r="C50" s="7" t="n">
         <v>9</v>
       </c>
@@ -2885,7 +3377,7 @@
           <t>15.2</t>
         </is>
       </c>
-      <c r="B52" s="15" t="n"/>
+      <c r="B52" s="19" t="n"/>
       <c r="C52" s="7" t="n">
         <v>3</v>
       </c>
@@ -2930,7 +3422,7 @@
           <t>15.3</t>
         </is>
       </c>
-      <c r="B53" s="15" t="n"/>
+      <c r="B53" s="19" t="n"/>
       <c r="C53" s="7" t="n">
         <v>3</v>
       </c>
@@ -2975,7 +3467,7 @@
           <t>15.4</t>
         </is>
       </c>
-      <c r="B54" s="15" t="n"/>
+      <c r="B54" s="19" t="n"/>
       <c r="C54" s="7" t="n">
         <v>3</v>
       </c>
@@ -3020,7 +3512,7 @@
           <t>15.5</t>
         </is>
       </c>
-      <c r="B55" s="15" t="n"/>
+      <c r="B55" s="19" t="n"/>
       <c r="C55" s="7" t="n">
         <v>3</v>
       </c>
@@ -3065,7 +3557,7 @@
           <t>15.6</t>
         </is>
       </c>
-      <c r="B56" s="15" t="n"/>
+      <c r="B56" s="16" t="n"/>
       <c r="C56" s="7" t="n">
         <v>3</v>
       </c>
@@ -3159,7 +3651,7 @@
           <t>16.2</t>
         </is>
       </c>
-      <c r="B58" s="15" t="n"/>
+      <c r="B58" s="19" t="n"/>
       <c r="C58" s="7" t="n">
         <v>3</v>
       </c>
@@ -3204,7 +3696,7 @@
           <t>16.3</t>
         </is>
       </c>
-      <c r="B59" s="15" t="n"/>
+      <c r="B59" s="19" t="n"/>
       <c r="C59" s="7" t="n">
         <v>3</v>
       </c>
@@ -3249,7 +3741,7 @@
           <t>16.4</t>
         </is>
       </c>
-      <c r="B60" s="15" t="n"/>
+      <c r="B60" s="19" t="n"/>
       <c r="C60" s="7" t="n">
         <v>3</v>
       </c>
@@ -3294,7 +3786,7 @@
           <t>16.5</t>
         </is>
       </c>
-      <c r="B61" s="15" t="n"/>
+      <c r="B61" s="19" t="n"/>
       <c r="C61" s="7" t="n">
         <v>3</v>
       </c>
@@ -3339,7 +3831,7 @@
           <t>16.6</t>
         </is>
       </c>
-      <c r="B62" s="15" t="n"/>
+      <c r="B62" s="16" t="n"/>
       <c r="C62" s="7" t="n">
         <v>3</v>
       </c>
@@ -3395,14 +3887,14 @@
 (선택 사항) 로터(드럼)와 패드(라이닝)의 두께와 무게를 측정합니다. 테스트 요청에 따라 고정 장치, 예압, 테스트 하드웨어, 마이크 및 가속도계를 철저히 검사합니다. 테스트 설정을 기록하기 위해 디지털 사진을 촬영합니다. 마이크와 가속도계 교정을 수행합니다. 7.3.3항에 따라 냉각 공기를 사용하여 배경 소음 점검을 수행합니다.</t>
         </is>
       </c>
-      <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="n"/>
-      <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="n"/>
-      <c r="H63" s="3" t="n"/>
-      <c r="I63" s="3" t="n"/>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="3" t="n"/>
+      <c r="D63" s="17" t="n"/>
+      <c r="E63" s="17" t="n"/>
+      <c r="F63" s="17" t="n"/>
+      <c r="G63" s="17" t="n"/>
+      <c r="H63" s="17" t="n"/>
+      <c r="I63" s="17" t="n"/>
+      <c r="J63" s="17" t="n"/>
+      <c r="K63" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -3412,7 +3904,6 @@
     <mergeCell ref="B36:B41"/>
     <mergeCell ref="B22:B28"/>
     <mergeCell ref="B44:B50"/>
-    <mergeCell ref="B14:B19"/>
     <mergeCell ref="B57:B62"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
@@ -3420,10 +3911,235 @@
     <mergeCell ref="C3:K3"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="I1:I2"/>
+    <mergeCell ref="B14:B19"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:J51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Figure 3 - Pressure profiles at increasing/decreasing pressure at constant brake speed; example shows the PP2.5 profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Time
+(seconds)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Brake pressure
+(kPa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Figure 4 - Speed profile SP2 at constant pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Table 2 - Speeds and times for speed profile SP2 at constant pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Time
+(seconds)</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Speed
+(km/h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C26" s="21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="C27" s="21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="21" t="n">
+        <v>23</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="21" t="n">
+        <v>26</v>
+      </c>
+      <c r="C29" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="21" t="n">
+        <v>36</v>
+      </c>
+      <c r="C30" s="21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="21" t="n">
+        <v>39</v>
+      </c>
+      <c r="C31" s="21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="21" t="n">
+        <v>49</v>
+      </c>
+      <c r="C32" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Figure 5 - Speed profile SP10 at constant pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Table 3 - Speeds and times for speed profile SP10 at constant pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Time
+(seconds)</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Speed
+(km/h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" s="22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C50" s="22" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C51" s="22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="B44:J44"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>